<commit_message>
Graficas de proceso de identificación
</commit_message>
<xml_diff>
--- a/datos/serie_empalmada_100obs.xlsx
+++ b/datos/serie_empalmada_100obs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20827"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARMANDOJRS107\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARMANDOJRS107\Desktop\Universidad Nando\Econometria 2\Poster-econometr-a-II-Serie-del-sector-financiero\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A51D95-F116-488D-92B4-8CF9FAD599FD}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71ACCB42-F94A-4293-907D-B9FC4E99DE6D}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="109">
   <si>
     <t>periodo</t>
   </si>
@@ -344,20 +344,62 @@
   </si>
   <si>
     <t>2025_IV</t>
+  </si>
+  <si>
+    <t>2025_I</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.00\ _P_t_s_-;\-* #,##0.00\ _P_t_s_-;_-* &quot;-&quot;??\ _P_t_s_-;_-@_-"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color indexed="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -396,16 +438,39 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="9">
+    <cellStyle name="Hipervínculo 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Millares 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
+    <cellStyle name="Millares 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
+    <cellStyle name="Normal 2 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 3 2" xfId="8" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
+    <cellStyle name="Normal 4" xfId="1" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
@@ -707,7 +772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D2:F105"/>
+  <dimension ref="D2:F106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="9.6640625" customWidth="1"/>
@@ -1828,21 +1893,21 @@
     </row>
     <row r="103" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D103" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E103" s="1">
-        <v>13259.484696990001</v>
-      </c>
-      <c r="F103" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E103" s="3">
+        <v>13139.131347857799</v>
+      </c>
+      <c r="F103" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="104" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D104" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E104" s="1">
-        <v>13470.782849166</v>
+        <v>13259.484696990001</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>25</v>
@@ -1850,12 +1915,23 @@
     </row>
     <row r="105" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D105" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E105" s="1">
+        <v>13470.782849166</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="106" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="D106" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E105" s="1">
+      <c r="E106" s="1">
         <v>13242.942832671</v>
       </c>
-      <c r="F105" s="1" t="s">
+      <c r="F106" s="1" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>